<commit_message>
fix(rd-jachymov): tvárnice ztraceného bednění → komplet (oprava chybného split)
Auto-splitter (Pattern 41) chybně rozkládal tvárnice ztraceného bednění:
- HSV2.003 patky horní → materiál-leg "Dodávka oceli S235" (chytil "IPE180"
  v popisu; přitom materiál jsou tvárnice ZB, ocel je samostatně HSV4.004)
- HSV3.002 stěna → materiál-leg "Pronájem bednění" (chytil "bednění" ve
  "ztraceného bednění"; ztracené bednění se NEpronajímá, zůstává v konstrukci)

Příčina: _KOMPLET má "tvárnic", ale popisy píší "tvarovek/tvarovky" +
"ztraceného bednění" → propadly do _SPLIT_RULES. Fix: _KOMPLET += "tvarov",
"ztracen" → tvárnice ZB zůstávají komplet (1 ÚRS položka m²/ks, jako reálné
zdivo z tvárnic ztraceného bednění). HSV2.003 popis/formula upřesněny
(6 sloupků = 12 tvárnic 300×300; zálivka C25/30 v HSV2.004). Atomic 374→371.

https://claude.ai/code/session_01FskzLAZkXgJAwuN2cQQEdx
</commit_message>
<xml_diff>
--- a/test-data/RD_Jachymov_dum/outputs/Vykaz_vymer_RD_Jachymov_KROS_format_2026-06-02_v3_final.xlsx
+++ b/test-data/RD_Jachymov_dum/outputs/Vykaz_vymer_RD_Jachymov_KROS_format_2026-06-02_v3_final.xlsx
@@ -17241,7 +17241,7 @@
       </c>
       <c r="E59" s="24" t="inlineStr">
         <is>
-          <t>Dvoustupňové patky pro IPE180 — horní část z tvarovek ztraceného bednění 300×300 mm × 6 ks</t>
+          <t>Patky parking horní část — zdivo z tvárnic ztraceného bednění 300×300 mm (lost formwork, zůstává v konstrukci), 6 patek á 300×300×500 mm</t>
         </is>
       </c>
       <c r="F59" s="23" t="inlineStr">
@@ -17283,7 +17283,7 @@
       <c r="D60" s="17" t="n"/>
       <c r="E60" s="29" t="inlineStr">
         <is>
-          <t>6 ks (= spodní, výkres D.1.1.02)</t>
+          <t>6 patek horní á 300×300×500 mm = 6 sloupků z tvárnic ZB 300×300 (á 2 řady po 250 = 12 tvárnic); zálivka C25/30 + výztuž samostatně (HSV2.004 / HSV3.003)</t>
         </is>
       </c>
       <c r="F60" s="17" t="n"/>
@@ -21954,7 +21954,7 @@
       <c r="F100" s="24" t="inlineStr"/>
       <c r="G100" s="24" t="inlineStr">
         <is>
-          <t>Dvoustupňové patky pro IPE180 — horní část z tvarovek ztraceného bedně</t>
+          <t xml:space="preserve">Patky parking horní část — zdivo z tvárnic ztraceného bednění 300×300 </t>
         </is>
       </c>
       <c r="H100" s="24" t="inlineStr">
@@ -28874,7 +28874,7 @@
       </c>
       <c r="D34" s="24" t="inlineStr">
         <is>
-          <t>Dvoustupňové patky pro IPE180 — horní část z tvarovek ztraceného bednění 300×300</t>
+          <t>Patky parking horní část — zdivo z tvárnic ztraceného bednění 300×300 mm (lost f</t>
         </is>
       </c>
       <c r="E34" s="24" t="inlineStr">

</xml_diff>